<commit_message>
Improve Sugar News editorial summaries
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-16.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-16.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -513,16 +513,16 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度糖厂披露糖厂运行和压榨安排，已披露具体事件方向但标题缺少数值。印度糖厂若增加开工或压榨，会加快当季食糖产出；若停产或延后开榨，则阶段性供应收紧。来源：BusinessLine（https://news.google.com/rss/articles/CBMi7wFBVV95cUxNTmZONlJGQWlkM1Z4a3pQRG1kaXVUbG5mUTh6RlhCVVZBeTg1dHNxVldaRG8yUl9kZHliYndQZ0wtbnhsOG9DdF9xTDJGMXItRm1HMEhZQzVjdDRHLXRvVHVOREoxYVdVZ3dfcWc0elY4a1JZanhrVG5wMzhuWlo2QjZjOURMVDlFclp5T0lnTWxBZFRqa3pyTlVmSGUzY29nX2RIdWpoNXREZVhHbEJLZlFCa0JWSTlLRk5oOHpNRnhJdFZTTmFHSlNidWJOcmJhQVJWM0ZNTG1qaEpSak5LMm0wc1pNNmthcDI3TEo5c9IB9gFBVV95cUxQMmdraHlHby1LeTRyR2lxREJsaHpFVTlXR0hOODVaSDg4ZGt6d194cHdZU0xyYnB5VUFUY3NkMHVOWVEtT1gtajFqbkhyN2U2LUEwQ1YyUFBZZEFrMHYtX2JVeTF6VERERVhYUFNoUVh6OVpnRGZXM3lDUTdxelpuOWdOYTRrQWR5eG5qb0l0Q0F4LXFqcXRlemFWQWR4dEl6TDNHVm04R2NZVTZIWjlXSXRpekM5YzF5V2lWSVF4QTVFQW1aREVkb3l3OEU2cjRGeXVEZ05sa2lzV3VpT3FILWtqLUR0T0xiTkE5VDBGcTVTSlM0alE?oc=5）</t>
+          <t>印度E20汽油推广将全国乙醇掺混率从2013/14年的约1.5%提高到2024/25年接近20%，原2030目标已提前到2025/26年，原料包括甘蔗衍生物、玉米和受损粮。E20扩大燃料乙醇需求；若新增供应由甘蔗汁、糖浆或B重糖蜜补充，可结晶蔗糖会转入乙醇而非食糖生产，减少食糖供应预期并支撑糖价。原文同时提到玉米和受损粮可参与供给，因此实际挤占食糖产量的幅度取决于后续原料结构。来源：ET Government（https://government.economictimes.indiatimes.com/blog/the-e20-debate-who-pays-the-price-for-indias-shift-towards-ethanol/133268836）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利空：糖厂运行、压榨能力或原料供应改善会提高食糖生产节奏，增加阶段性供应。</t>
+          <t>利多：E20扩大燃料乙醇需求；若新增供应由甘蔗汁、糖浆或B重糖蜜补充，可结晶蔗糖会转入乙醇而非食糖生产，减少食糖供应预期并支撑糖价。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="180" customHeight="1" s="2">
+    <row r="3" ht="174.15" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -530,12 +530,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构公布乙醇掺混或燃料政策，指标包括1KL、E20。若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量。来源：ET Government（https://news.google.com/rss/articles/CBMiyAFBVV95cUxPcXA2ZWE0Q0Z5dW1kWjJCT2hpYW5JVEFQY2JEVl9weEEzSmJ1WFBxaThrcTBuR3FfQWVnTHJpaWtZeTRFLXRpbV95aTkyMkdtUlZVVmpMUzZKZV90WlRDSGxldDF6aFBHVUIzckRjcTIzUnlVaEJpdFFzZ3BsVXh0M25ibjFlUDBJYXJ6YWJTY2JwcW50RTd3aFFKY2FNM0RtUzVBRTlBNVBPWVU0X3VZS1VseDJTVVZiZ3dNejA0a010NXlERjZZetIBzgFBVV95cUxObGhpeDYtb0V0a01oc2o5SlAtM0xJNG1oRjVJQlZtVTE3cXlFdXRHOGhBQWpJbEtBZlkxUnpKOGNHR0ZPY0xJNnpnOTRhZ3RzQm1Ebk1UdDdrQjNnd0Z6TmVQek9pMDF2WDZrWDd6U25kNEJKckl4bUt5WElwQmQ3MVYyc3ZLcEktbVZteGNtSkZDN0Jacl9XcVc4amFVQTBNZTlhdWx3UV9aTE1KLVZxVEljbHM5NE85YnpudXgtZkppWU50NjQ2Yklka2Vrdw?oc=5）</t>
+          <t>周末延续消息：印度食品和公共分配部下属糖与植物油局要求所有糖厂在售糖后7日内让买方提离糖库存，原因是部分糖厂库存高于P2表申报量或销售低于月度配额，指令执行至2026年11月30日。该要求会压缩糖厂把已售糖留在厂内制造阶段性短缺的空间，加快库存进入贸易和消费环节，增加印度国内可流通糖源并压制现货糖价。来源：ChiniMandi（https://www.chinimandi.com/government-directs-sugar-mills-to-clear-stock-within-seven-days-of-sale/）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利多：若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量，从而减少食糖供应预期并支撑糖价。</t>
+          <t>利空：印度要求糖厂售糖后7日内清出库存，加快已售食糖进入贸易和消费环节，增加国内可流通糖源并压制现货糖价。</t>
         </is>
       </c>
     </row>
@@ -547,16 +547,16 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>印度政府披露糖厂运行和压榨安排，已披露具体事件方向但标题缺少数值。印度糖厂若增加开工或压榨，会加快当季食糖产出；若停产或延后开榨，则阶段性供应收紧。来源：ChiniMandi（https://news.google.com/rss/articles/CBMioAFBVV95cUxPZDQwWnpoWmNqUGw2SkkwYzlyekFlVkFGT0tMZHRfamRsZGxQZ2cyRE5taGUwNDVqcE16MVlZZU9KcS1NanpJS3E2amd0OXVqd1pfaHVCd2lRTmFIVC04U25qbk5MdFBHZDFCdldjakxrY2pPWkVxcTJEMFJJNnBmcHpWRy0wejRnX1NwTXlBT2xmU3pWRlJWdE1WWENzUVpX?oc=5）</t>
+          <t>印度糖厂正由单一制糖转向综合生物炼厂，印度已在2025年达到汽油20%乙醇掺混，政府支持把甘蔗基蒸馏厂改为可同时使用糖基原料、玉米和碎米的多原料装置。多原料装置会扩大糖厂乙醇和副产品收入，但玉米、碎米可在甘蔗淡季替代部分糖蜜或糖浆制醇需求，降低对可结晶糖源的直接挤占。原文没有给出当期甘蔗压榨量或食糖产量调整，对糖价按中性处理。来源：BusinessLine（https://www.thehindubusinessline.com/economy/agri-business/from-sugar-mill-to-biorefinery-the-next-transformation-of-indias-sugar-industry/article71346916.ece）。影响：中性</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>利空：糖厂运行、压榨能力或原料供应改善会提高食糖生产节奏，增加阶段性供应。</t>
+          <t>中性：多原料制醇扩大乙醇收入，但玉米、碎米替代部分糖蜜或糖浆需求时会降低对可结晶糖源的挤占；原文未调整当期食糖产量或库存，对糖价方向暂不单边。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="110.35" customHeight="1" s="2">
+    <row r="5" ht="98.80000000000001" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>泰国</t>
@@ -564,29 +564,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>泰国气象局预报（2026-08-16），那空沙旺、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
+          <t>泰国气象局预报8月16日那空沙旺、北碧等主要甘蔗产区有雷阵雨并伴有局地大雨。泰国处于甘蔗生长期，降雨有利于补充产区土壤水分、改善墒情并提高后期甘蔗单产和食糖供应预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118.05" customHeight="1" s="2">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>中国</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
+          <t>利空：泰国甘蔗生长期降雨有利于补充土壤水分、改善墒情并促进单产形成，从而增加未来甘蔗及食糖供应预期。</t>
         </is>
       </c>
     </row>

</xml_diff>